<commit_message>
Unify RCM A–N terminology and tighten control wording
Apply consistent internal-control column logic through 控制現況
(風險因素→風險描述→控制目標→控制活動→現況), standardize terms
(資訊單位／資訊人員／帳號／正式作業環境／預防性／偵測性等), trim
verbose interview phrasing, and align 控制現況 to each control.
Edited cells marked in red; columns right of 控制現況 untouched.

Co-authored-by: Lawr3nc3Ku01118 <lawrencekuo1118@gmail.com>
</commit_message>
<xml_diff>
--- a/whalechip-rcm/鯨銘科技_資訊循環_RCM v1 (0820).xlsx
+++ b/whalechip-rcm/鯨銘科技_資訊循環_RCM v1 (0820).xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="169" formatCode="0.000_);[Red]\(0.000\)"/>
     <numFmt numFmtId="170" formatCode="0.0000_);[Red]\(0.0000\)"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="32">
     <font>
       <name val="Calibri"/>
       <charset val="136"/>
@@ -221,6 +221,12 @@
     </font>
     <font>
       <name val="Arial Unicode MS"/>
+      <color rgb="FFFF0000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial Unicode MS"/>
+      <b val="1"/>
       <color rgb="FFFF0000"/>
       <sz val="10"/>
     </font>
@@ -591,7 +597,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -796,6 +802,33 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="21" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1488,9 +1521,9 @@
           <t>控制頻率</t>
         </is>
       </c>
-      <c r="N2" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">控制現況描述 </t>
+      <c r="N2" s="70" t="inlineStr">
+        <is>
+          <t>控制現況描述</t>
         </is>
       </c>
       <c r="O2" s="44" t="inlineStr">
@@ -1561,9 +1594,9 @@
           <t>職能分工</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>使用者充當資訊系統開發者，導致該系統犧牲安全性以換取效能提升或被偏廢</t>
+      <c r="E3" s="61" t="inlineStr">
+        <is>
+          <t>使用者兼任資訊系統開發，可能犧牲安全性以換取效能或功能偏廢</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
@@ -1606,9 +1639,9 @@
           <t>持續</t>
         </is>
       </c>
-      <c r="N3" s="24" t="inlineStr">
-        <is>
-          <t>公司資訊部門共配置兩名人員（資訊主管/資訊人員）。資訊主管主要負責與研發單位配合，相關系統伺服器管理、雲端服務維運及公司帳號建立與管理；資訊人員則負責網路與硬體設備維護、使用者權限管理及部分系統開發作業。</t>
+      <c r="N3" s="71" t="inlineStr">
+        <is>
+          <t>資訊單位共兩人（主管／資訊人員）。主管負責與研發配合、伺服器及雲端維運、帳號建立與管理；資訊人員負責網路與硬體維護、使用者權限管理及部分系統開發。</t>
         </is>
       </c>
       <c r="O3" s="24" t="inlineStr">
@@ -1651,9 +1684,9 @@
           <t>職能分工</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>資訊人員權限過大致犧牲系統安全性以換取維護便利性</t>
+      <c r="E4" s="61" t="inlineStr">
+        <is>
+          <t>資訊人員權限過大，可能犧牲系統安全性以換取維護便利</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
@@ -1676,9 +1709,9 @@
           <t>EC-101-02</t>
         </is>
       </c>
-      <c r="J4" s="39" t="inlineStr">
-        <is>
-          <t>公司應明訂資訊單位之組織任務及功能職掌，並確保工作職責均有明確劃分，且不相容之職務不得由同一人兼任。</t>
+      <c r="J4" s="72" t="inlineStr">
+        <is>
+          <t>公司應明訂資訊單位組織任務及功能職掌，劃分工作職責，且不相容職務不得由同一人兼任。</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -1696,9 +1729,9 @@
           <t>持續</t>
         </is>
       </c>
-      <c r="N4" s="24" t="inlineStr">
-        <is>
-          <t>依照公司預算管理辦法執行，係由財務部門主導預算彙整流程，提供制式化表單向資訊單位蒐集年度需求後，由資訊部門填列相關費用（目前以維修費用為主），經營運長核准後由財務部門彙整。</t>
+      <c r="N4" s="71" t="inlineStr">
+        <is>
+          <t>資訊單位內部職掌已大致分工，惟不相容職務之細項區隔及書面規範待確認。</t>
         </is>
       </c>
       <c r="O4" s="24" t="inlineStr">
@@ -1751,9 +1784,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>重要資訊活動方向與公司目標一致且資金充裕不受營運表現影響</t>
+      <c r="H5" s="61" t="inlineStr">
+        <is>
+          <t>重要資訊活動方向與公司目標一致，並經適當資源核配</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -1761,9 +1794,9 @@
           <t>EC-101-03</t>
         </is>
       </c>
-      <c r="J5" s="39" t="inlineStr">
-        <is>
-          <t>資訊單位研擬短、中、長期資訊計劃及年度預算，應經相關利害關係人參與評估，並取得高階管理人員核准。</t>
+      <c r="J5" s="72" t="inlineStr">
+        <is>
+          <t>資訊單位研擬短、中、長期資訊計畫及年度預算，應經相關利害關係人評估，並取得高階管理人員核准。</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -1781,9 +1814,9 @@
           <t>每年</t>
         </is>
       </c>
-      <c r="N5" s="24" t="inlineStr">
-        <is>
-          <t>目前資訊預算內容較偏向維護、營運性質，尚未明確涵蓋中長期資訊發展規劃。</t>
+      <c r="N5" s="71" t="inlineStr">
+        <is>
+          <t>資訊年度預算由財務部門以制式表單蒐集需求，資訊單位填列費用（目前以維修為主），經營運長核准後由財務彙整。預算內容偏維運，尚未涵蓋中長期資訊發展規劃。</t>
         </is>
       </c>
       <c r="O5" s="24" t="n"/>
@@ -1821,9 +1854,9 @@
           <t>代理人訓練</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>資訊系統維運中斷或異常事件無法及時處理</t>
+      <c r="E6" s="61" t="inlineStr">
+        <is>
+          <t>資訊系統維運中斷或異常時，無法及時處理</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
@@ -1846,9 +1879,9 @@
           <t>EC-101-04</t>
         </is>
       </c>
-      <c r="J6" s="39" t="inlineStr">
-        <is>
-          <t>資訊單位應落實職務代理人交叉訓練，以加強人員備援能力與偵防弊端。</t>
+      <c r="J6" s="72" t="inlineStr">
+        <is>
+          <t>資訊單位應落實職務代理人交叉訓練，強化備援能力。</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1866,9 +1899,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N6" s="24" t="inlineStr">
-        <is>
-          <t>資訊部門代理人制度，由兩位人員互為代理。另在人員訓練方面，目前曾參與Office 365及ISO 27001相關課程。</t>
+      <c r="N6" s="71" t="inlineStr">
+        <is>
+          <t>資訊單位兩人互為代理；曾參與 Office 365 及 ISO 27001 相關課程。</t>
         </is>
       </c>
       <c r="O6" s="24" t="inlineStr">
@@ -1935,9 +1968,9 @@
           <t>EC-101-05</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>公司應於員工到職或相關教育訓練時，向員工宣導智慧財產權相關法令及公司規範，並要求員工遵循不得侵害公司或第三方智慧財產權之規定。</t>
+      <c r="J7" s="61" t="inlineStr">
+        <is>
+          <t>公司應於員工到職或教育訓練時宣導智慧財產權法令及公司規範，並要求員工遵循。</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2040,10 +2073,9 @@
           <t>持續</t>
         </is>
       </c>
-      <c r="N8" s="51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">公司已訂定「系統開發及程式修改控制作業」，規範各單位提出系統或程式修改需求時，應填具「系統申請/修改單」或「報表程式需求申請單」，經使用單位主管簽核後送交資訊單位；資訊單位取得申請文件及需求內容後，對程式修改需求執行可行性評估及核准，經核准後始進行自行修改或委外修改。程式修改完成後，由資訊單位先行測試，測試無誤後交由使用單位確認驗收，並於測試及驗收無誤後始得上線使用；相關申請文件由資訊單位編號存檔備查，並記錄系統文件修改內容，以確保系統程式修改均依變更申請、測試、驗收、核准及部署程序執行。
-</t>
+      <c r="N8" s="73" t="inlineStr">
+        <is>
+          <t>已訂定「系統開發及程式修改控制作業」。需求單位填具「系統申請/修改單」或「報表程式需求申請單」，經使用單位主管簽核後送資訊單位；資訊單位評估核准後自行或委外修改，完成測試並經使用單位驗收後始得上線；申請文件由資訊單位編號存檔。</t>
         </is>
       </c>
       <c r="O8" s="3" t="inlineStr">
@@ -2081,9 +2113,9 @@
           <t>系統變更管理</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>系統版本或架構改動錯誤，導致系統功能異常、交易處理失敗、報表產出錯誤或批次作業中斷</t>
+      <c r="E9" s="61" t="inlineStr">
+        <is>
+          <t>系統版本或架構變更錯誤，導致功能異常、交易失敗、報表錯誤或批次中斷</t>
         </is>
       </c>
       <c r="F9" s="1" t="inlineStr">
@@ -2126,9 +2158,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N9" s="52" t="inlineStr">
-        <is>
-          <t>目前大多透過會議口頭討論執行，並無正式的書面核准紀錄。</t>
+      <c r="N9" s="60" t="inlineStr">
+        <is>
+          <t>多以會議口頭討論執行，無書面核准紀錄。</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
@@ -2166,9 +2198,9 @@
           <t>資料庫結構變更管理</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>資料庫結構改動錯誤，導致應用系統功能異常、資料處理錯誤、報表資訊不正確、資料完整性受損或系統中斷</t>
+      <c r="E10" s="61" t="inlineStr">
+        <is>
+          <t>資料庫結構變更錯誤，導致應用異常、資料錯誤、報表不正確、完整性受損或系統中斷</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -2211,14 +2243,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N10" s="53" t="inlineStr">
-        <is>
-          <t>1.資料庫變更：原則上不允許，惟曾因組織調整而執行的大批量部門編號異動，係由資訊人員直接在後台執行，該作業並無正式書面核准紀錄。
-2.稽核軌跡：前 Office 365 具備內建監控功能，但核心系統如 ERP 則明確表示目前無存取監控機制，目前亦無詳細的變更日誌（Change Log）或稽核軌跡可供查核。
-3.權限設定：目前同仁均配發獨立帳號與密碼，存取權限係依據人事單位的組織架構圖進行設定與鎖定。
-4.經應用程式修改資料庫：未提及
-5.資料庫備份：系統具備每日凌晨自動備份機制，並留存 90 個歷史版本。
-6.迅速取得備援資料庫：未提及</t>
+      <c r="N10" s="60" t="inlineStr">
+        <is>
+          <t>資料庫結構異動原則上不允許；曾因組織調整由資訊人員於後台批次異動部門編號，無書面核准紀錄。</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -2260,9 +2287,9 @@
           <t>環境區隔控制</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>未經驗證之系統變更直接影響正式作業環境，造成系統異常、資料錯誤或營運中斷</t>
+      <c r="E11" s="61" t="inlineStr">
+        <is>
+          <t>未經驗證之系統變更直接影響正式作業環境，造成異常、資料錯誤或營運中斷</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
@@ -2285,9 +2312,9 @@
           <t>EC-102-04</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>系統應區分正式作業環境與非正式作業環境；系統變更應於非正式環境完成測試。</t>
+      <c r="J11" s="61" t="inlineStr">
+        <is>
+          <t>系統應區分正式作業環境與非正式作業環境；系統變更應於非正式作業環境完成測試。</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -2305,9 +2332,9 @@
           <t>持續</t>
         </is>
       </c>
-      <c r="N11" s="52" t="inlineStr">
-        <is>
-          <t>目前公司針對自研之應用系統（如績效考核系統）係直接於正式環境介面進行功能開發與使用者驗收，尚未建置與正式作業環境完全區隔之獨立測試環境。</t>
+      <c r="N11" s="60" t="inlineStr">
+        <is>
+          <t>自研應用系統（如績效考核系統）係於正式作業環境介面開發並驗收，尚未建置獨立測試環境。</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr">
@@ -2345,9 +2372,9 @@
           <t>系統測試設計</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>未妥善測試之新開發系統或修改後程式造成運作出現異常，導致營運受影響或中斷</t>
+      <c r="E12" s="61" t="inlineStr">
+        <is>
+          <t>新開發或修改後程式未經妥善測試，導致營運異常或中斷</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
@@ -2370,9 +2397,9 @@
           <t>EC-102-05</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>資訊單位於系統開發或程式修改過程中，應依變更內容規劃適當測試方式，視情況包含系統測試、單元測試、介面測試、平行測試、容量測試及使用者接受程度測試等。</t>
+      <c r="J12" s="61" t="inlineStr">
+        <is>
+          <t>資訊單位於系統開發或程式修改時，應依變更內容規劃適當測試（含系統、單元、介面、平行、容量及使用者接受測試等）。</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -2390,9 +2417,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N12" s="52" t="inlineStr">
-        <is>
-          <t>目前應用系統（如績效考核系統）之變更測試係於開發完成後，由資訊人員直接邀請使用者在正式環境介面進行功能驗收與口頭討論。</t>
+      <c r="N12" s="60" t="inlineStr">
+        <is>
+          <t>應用系統（如績效考核系統）開發完成後，由資訊人員邀請使用者於正式作業環境介面進行功能驗收與口頭討論。</t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr">
@@ -2430,9 +2457,9 @@
           <t>測試資料管理</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>測試因使用之資料不完整或欠缺代表性而無效</t>
+      <c r="E13" s="61" t="inlineStr">
+        <is>
+          <t>測試資料不完整或欠缺代表性，致使測試無效</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">
@@ -2455,9 +2482,9 @@
           <t>EC-102-06</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>應用系統測試應使用完整且具代表性之測試資料，而非使用實際作業環境之資料。</t>
+      <c r="J13" s="61" t="inlineStr">
+        <is>
+          <t>應用系統測試應使用完整且具代表性之測試資料，不得直接使用正式作業環境資料。</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -2538,14 +2565,14 @@
           <t>系統程式修改控制作業</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>正式部署 / 過版</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>系統變更未考量營運單位時程安排，使實際營運作業受影響或被迫中斷</t>
+      <c r="D14" s="61" t="inlineStr">
+        <is>
+          <t>正式部署／過版</t>
+        </is>
+      </c>
+      <c r="E14" s="61" t="inlineStr">
+        <is>
+          <t>系統變更未配合營運單位時程，影響或中斷既有作業</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr">
@@ -2558,9 +2585,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>系統正式環境之變更經適當規劃及管理而不影響既有作業流程</t>
+      <c r="H14" s="61" t="inlineStr">
+        <is>
+          <t>正式作業環境變更經適當規劃，不影響既有作業流程</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -2568,9 +2595,9 @@
           <t>EC-102-07</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>於正式環境變動應用系統時，資訊單位應配合相關單位時程執行，避免影響其既有作業流程。</t>
+      <c r="J14" s="61" t="inlineStr">
+        <is>
+          <t>於正式作業環境變更應用系統時，資訊單位應配合相關單位時程執行，避免影響既有作業。</t>
         </is>
       </c>
       <c r="K14" s="9" t="inlineStr">
@@ -2651,14 +2678,14 @@
           <t>系統程式修改控制作業</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>正式部署 / 過版</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>系統過版後無法檢視部署前後差異作為未來改善依據</t>
+      <c r="D15" s="61" t="inlineStr">
+        <is>
+          <t>正式部署／過版</t>
+        </is>
+      </c>
+      <c r="E15" s="61" t="inlineStr">
+        <is>
+          <t>系統過版後無法比對部署前後差異，不利復原與改善</t>
         </is>
       </c>
       <c r="F15" s="1" t="inlineStr">
@@ -2671,9 +2698,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>提升系統過版失敗之復原可能性</t>
+      <c r="H15" s="61" t="inlineStr">
+        <is>
+          <t>系統過版失敗時具備復原可能性</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -2701,9 +2728,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N15" s="52" t="inlineStr">
-        <is>
-          <t>績效考績系統更新過板後留下100個程式碼舊版本。</t>
+      <c r="N15" s="60" t="inlineStr">
+        <is>
+          <t>績效考核系統過版後保留約 100 個程式舊版本。</t>
         </is>
       </c>
       <c r="O15" s="3" t="n"/>
@@ -2732,14 +2759,14 @@
           <t>系統程式修改控制作業</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>正式部署 / 過版</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>系統過版出現重大異常而未能回復原狀</t>
+      <c r="D16" s="61" t="inlineStr">
+        <is>
+          <t>正式部署／過版</t>
+        </is>
+      </c>
+      <c r="E16" s="61" t="inlineStr">
+        <is>
+          <t>系統過版發生重大異常而未能回復原狀</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr">
@@ -2752,9 +2779,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>系統過版不影響既有作業流程及系統正常運作</t>
+      <c r="H16" s="61" t="inlineStr">
+        <is>
+          <t>系統過版不影響既有作業及系統正常運作</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -2762,9 +2789,9 @@
           <t>EC-102-09</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t>系統變更正式部署後如發生重大異常情形，資訊人員應依既定程序回復至前一正常版本。</t>
+      <c r="J16" s="61" t="inlineStr">
+        <is>
+          <t>系統變更正式部署後如發生重大異常，資訊人員應依既定程序回復至前一正常版本。</t>
         </is>
       </c>
       <c r="K16" s="9" t="inlineStr">
@@ -2818,9 +2845,9 @@
           <t>使用者驗收</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>變更後系統或程式功能不符合使用者需求</t>
+      <c r="E17" s="61" t="inlineStr">
+        <is>
+          <t>變更後系統或程式不符合使用者需求</t>
         </is>
       </c>
       <c r="F17" s="1" t="inlineStr">
@@ -2843,9 +2870,9 @@
           <t>EC-102-10</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>變更後應用系統，應經資訊單位與使用單位驗收通過後，始能正式上線。</t>
+      <c r="J17" s="61" t="inlineStr">
+        <is>
+          <t>變更後應用系統應經資訊單位與使用單位驗收通過後，始得正式上線。</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -2863,9 +2890,9 @@
           <t>持續</t>
         </is>
       </c>
-      <c r="N17" s="52" t="inlineStr">
-        <is>
-          <t>程式修改作業主要透過與需求單位會議討論後由資訊人員直接執行，並由使用者於正式介面上進行功能驗收。</t>
+      <c r="N17" s="60" t="inlineStr">
+        <is>
+          <t>程式修改多經與需求單位會議討論後由資訊人員執行，並由使用者於正式作業環境介面驗收。</t>
         </is>
       </c>
       <c r="O17" s="3" t="inlineStr">
@@ -2898,14 +2925,14 @@
           <t>系統程式修改控制作業</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>教育訓練 / 正式上線</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>使用者無法適應變更後系統或程式功能而影響營運作業</t>
+      <c r="D18" s="61" t="inlineStr">
+        <is>
+          <t>教育訓練／正式上線</t>
+        </is>
+      </c>
+      <c r="E18" s="61" t="inlineStr">
+        <is>
+          <t>使用者無法適應變更後系統功能，影響營運作業</t>
         </is>
       </c>
       <c r="F18" s="1" t="inlineStr">
@@ -2918,9 +2945,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="H18" s="40" t="inlineStr">
-        <is>
-          <t>建置後系統或程式皆能被使用者順利使用</t>
+      <c r="H18" s="74" t="inlineStr">
+        <is>
+          <t>建置後系統或程式可被使用者正確使用</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -2928,9 +2955,9 @@
           <t>EC-102-11</t>
         </is>
       </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>新系統建置完成後，由資訊單位或系統供應商辦理使用者教育訓練及操作說明，協助使用者瞭解系統功能及作業流程。</t>
+      <c r="J18" s="61" t="inlineStr">
+        <is>
+          <t>新系統建置完成後，由資訊單位或系統供應商辦理使用者教育訓練及操作說明。</t>
         </is>
       </c>
       <c r="K18" s="9" t="inlineStr">
@@ -2948,9 +2975,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N18" s="52" t="inlineStr">
-        <is>
-          <t>外購系統（如電子簽核、文管系統）建置時由廠商提供輔導課程與講解，而自研系統（如績效考核系統）則視需求召集使用者進行口頭操作說明與示範。</t>
+      <c r="N18" s="60" t="inlineStr">
+        <is>
+          <t>外購系統（如電子簽核、文管）由廠商提供輔導課程；自研系統（如績效考核系統）視需求召集使用者口頭說明與示範。</t>
         </is>
       </c>
       <c r="O18" s="3" t="inlineStr">
@@ -2988,9 +3015,9 @@
           <t>系統變更管理</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>系統變更專案超出預算與人力時間資源限制</t>
+      <c r="E19" s="61" t="inlineStr">
+        <is>
+          <t>系統變更專案超出預算、人力或時程限制</t>
         </is>
       </c>
       <c r="F19" s="1" t="inlineStr">
@@ -3033,9 +3060,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N19" s="52" t="inlineStr">
-        <is>
-          <t>目前大多透過會議口頭討論執行，並無正式的書面核准紀錄。</t>
+      <c r="N19" s="60" t="inlineStr">
+        <is>
+          <t>多以會議口頭討論追蹤，無書面核准或結案覆核紀錄。</t>
         </is>
       </c>
       <c r="O19" s="3" t="inlineStr">
@@ -3073,9 +3100,9 @@
           <t>系統文書管理</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>系統重要文書因久未更新而無法被新進或他單位人員參照使用</t>
+      <c r="E20" s="61" t="inlineStr">
+        <is>
+          <t>系統重要文書久未更新，無法供新進或其他單位人員參照</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
@@ -3098,9 +3125,9 @@
           <t>EC-103-01</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>公司應評估實際作業需求，編製重要系統之作業說明文書，並取得資訊權責主管適當核准。</t>
+      <c r="J20" s="61" t="inlineStr">
+        <is>
+          <t>公司應依實際作業需求編製重要系統作業說明文書，並取得資訊單位主管核准。</t>
         </is>
       </c>
       <c r="K20" s="9" t="inlineStr">
@@ -3118,9 +3145,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N20" s="51" t="inlineStr">
-        <is>
-          <t>自研之應用程式或小工具在開發完成上線前，其作業說明文件並未經過資訊主管或管理階層的正式核准程序。</t>
+      <c r="N20" s="73" t="inlineStr">
+        <is>
+          <t>自研應用程式或小工具上線前，作業說明文件未經資訊單位主管或管理階層正式核准。</t>
         </is>
       </c>
       <c r="O20" s="3" t="n"/>
@@ -3149,14 +3176,14 @@
           <t>編製系統文書之控制作業</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>版本管理 / 制度與程序</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>系統文書版本管理紊亂，使員工難以遵循，影響公司營運作業效率</t>
+      <c r="D21" s="61" t="inlineStr">
+        <is>
+          <t>版本管理／制度與程序</t>
+        </is>
+      </c>
+      <c r="E21" s="61" t="inlineStr">
+        <is>
+          <t>系統文書版本管理紊亂，員工難以遵循，影響作業效率</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr">
@@ -3179,9 +3206,9 @@
           <t>EC-103-02</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t>公司應將所有系統文書納入版本控管，明訂文件建立、修訂、核准、發布、保存及使用權限管理機制；系統文書異動時，應依公司安全管制及版本變更程序辦理，並留存版本變更紀錄。</t>
+      <c r="J21" s="61" t="inlineStr">
+        <is>
+          <t>系統文書應納入版本控管，明訂建立、修訂、核准、發布、保存及使用權限；異動時依程序辦理並留存版本變更紀錄。</t>
         </is>
       </c>
       <c r="K21" s="9" t="inlineStr">
@@ -3199,9 +3226,9 @@
           <t>持續</t>
         </is>
       </c>
-      <c r="N21" s="52" t="inlineStr">
-        <is>
-          <t>外購軟體無說明書，會直接來開輔導課程；自研程式有文件（說明書），但因為目前都是很小的程式，所以不會有核准流程。</t>
+      <c r="N21" s="60" t="inlineStr">
+        <is>
+          <t>外購軟體多以廠商輔導課程代替說明書；自研程式有說明文件，惟規模較小，未建立核准流程。</t>
         </is>
       </c>
       <c r="O21" s="3" t="inlineStr">
@@ -3239,9 +3266,9 @@
           <t>系統文書管理</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>使用者參照錯誤版本之說明文件或手冊，造成系統功能被不當操作使用</t>
+      <c r="E22" s="61" t="inlineStr">
+        <is>
+          <t>使用者參照錯誤版本之說明文件，造成系統操作不當</t>
         </is>
       </c>
       <c r="F22" s="1" t="inlineStr">
@@ -3254,9 +3281,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>使用者皆能取得新系統功能完整且正確之操作支援或說明</t>
+      <c r="H22" s="61" t="inlineStr">
+        <is>
+          <t>使用者可取得與現行功能一致之操作說明</t>
         </is>
       </c>
       <c r="I22" s="9" t="inlineStr">
@@ -3264,9 +3291,9 @@
           <t>EC-103-03</t>
         </is>
       </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>新增系統功能時，相關文件或手冊應適時更新、經資訊主管審閱無誤後，始得發布。</t>
+      <c r="J22" s="61" t="inlineStr">
+        <is>
+          <t>新增系統功能時，相關文件或手冊應同步更新，經資訊單位主管審閱後始得發布。</t>
         </is>
       </c>
       <c r="K22" s="9" t="inlineStr">
@@ -3284,9 +3311,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N22" s="52" t="inlineStr">
-        <is>
-          <t>目前針對自研之應用程式（如績效考核系統）雖具備基礎操作說明，但係由資訊人員自行編製後即配合程式上線，且後續新增功能或異動時亦未配合同步修訂相關手冊，亦未經過資訊主管之正式審核程序。</t>
+      <c r="N22" s="60" t="inlineStr">
+        <is>
+          <t>自研應用（如績效考核系統）有基礎操作說明，由資訊人員編製後即隨程式上線；功能異動時未同步修訂，亦未經資訊單位主管審閱。</t>
         </is>
       </c>
       <c r="O22" s="3" t="inlineStr">
@@ -3319,14 +3346,14 @@
           <t>編製系統文書之控制作業</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>系統文書管理 / 委外資訊服務</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>使用者無法適應新系統或程式功能而影響營運作業</t>
+      <c r="D23" s="61" t="inlineStr">
+        <is>
+          <t>系統文書管理／委外資訊服務</t>
+        </is>
+      </c>
+      <c r="E23" s="61" t="inlineStr">
+        <is>
+          <t>委外或購置系統缺乏完整操作支援，使用者無法正確使用</t>
         </is>
       </c>
       <c r="F23" s="1" t="inlineStr">
@@ -3349,9 +3376,9 @@
           <t>EC-103-04</t>
         </is>
       </c>
-      <c r="J23" s="3" t="inlineStr">
-        <is>
-          <t>委外開發或購置之系統，應要求廠商提供相關使用者操作手冊、系統設定文件手冊及客製化原始程式碼文件等。</t>
+      <c r="J23" s="61" t="inlineStr">
+        <is>
+          <t>委外開發或購置之系統，應要求廠商提供使用者操作手冊、系統設定文件及客製化原始程式碼文件等。</t>
         </is>
       </c>
       <c r="K23" s="9" t="inlineStr">
@@ -3369,9 +3396,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N23" s="51" t="inlineStr">
-        <is>
-          <t>公司目前針對外購之重要系統，如「電子簽核系統」、「ERP系統」及「文管系統」，主要由系統廠商提供輔導課程、操作講解及相關使用說明，以協助使用者瞭解系統功能及操作方式。</t>
+      <c r="N23" s="73" t="inlineStr">
+        <is>
+          <t>外購重要系統（電子簽核、ERP、文管）由廠商提供輔導課程、操作講解及使用說明。</t>
         </is>
       </c>
       <c r="O23" s="3" t="n"/>
@@ -3400,14 +3427,14 @@
           <t>程式及資料之存取控制作業</t>
         </is>
       </c>
-      <c r="D24" s="56" t="inlineStr">
-        <is>
-          <t>密碼管理 / 特權帳號管理</t>
-        </is>
-      </c>
-      <c r="E24" s="57" t="inlineStr">
-        <is>
-          <t>未經授權人員透過系統管理權限造使系統設定遭變更、資料遭不當存取或安全機制遭停用</t>
+      <c r="D24" s="61" t="inlineStr">
+        <is>
+          <t>密碼管理／特權帳號管理</t>
+        </is>
+      </c>
+      <c r="E24" s="75" t="inlineStr">
+        <is>
+          <t>未經授權人員藉系統管理權限變更設定、不當存取資料或停用安全機制</t>
         </is>
       </c>
       <c r="F24" s="58" t="inlineStr">
@@ -3430,9 +3457,9 @@
           <t>EC-104-01</t>
         </is>
       </c>
-      <c r="J24" s="56" t="inlineStr">
-        <is>
-          <t>各類資訊系統之管理員、超級使用者及其他特權帳號，不得沿用原廠預設帳號及密碼；系統安裝或設置完成後，應立即變更預設密碼，並依實際需要停用、更名或限制使用預設帳號。</t>
+      <c r="J24" s="61" t="inlineStr">
+        <is>
+          <t>各類資訊系統之管理員、超級使用者及其他特權帳號，不得沿用原廠預設帳號及密碼；安裝或設置完成後應立即變更預設密碼，並視需要停用、更名或限制預設帳號。</t>
         </is>
       </c>
       <c r="K24" s="55" t="inlineStr">
@@ -3490,9 +3517,9 @@
           <t>特權帳號管理</t>
         </is>
       </c>
-      <c r="E25" s="58" t="inlineStr">
-        <is>
-          <t>特權帳號及其權限遭未經授權人員使用或逾越維運需求存取系統、修改設定及處理資料</t>
+      <c r="E25" s="61" t="inlineStr">
+        <is>
+          <t>特權帳號或其權限遭未經授權使用，或逾越維運需求存取系統、修改設定及處理資料</t>
         </is>
       </c>
       <c r="F25" s="58" t="inlineStr">
@@ -3537,7 +3564,7 @@
       </c>
       <c r="N25" s="60" t="inlineStr">
         <is>
-          <t>按公司政策"XXX"，針對績效考績系統，原則上為IT人員負責。</t>
+          <t>特權帳號原則由資訊人員管理（政策名稱待確認）；建立、異動及停用之核准軌跡未提及。</t>
         </is>
       </c>
       <c r="O25" s="61" t="inlineStr">
@@ -3575,9 +3602,9 @@
           <t>特權帳號覆核</t>
         </is>
       </c>
-      <c r="E26" s="58" t="inlineStr">
-        <is>
-          <t>重要應用系統之特權帳號及權限遭歸屬不明或已無使用需求之帳號不當使用，或持續保有逾越維運需求之權限</t>
+      <c r="E26" s="61" t="inlineStr">
+        <is>
+          <t>應用系統特權帳號歸屬不明、已無需求或權限過大</t>
         </is>
       </c>
       <c r="F26" s="58" t="inlineStr">
@@ -3600,9 +3627,9 @@
           <t>EC-104-03</t>
         </is>
       </c>
-      <c r="J26" s="58" t="inlineStr">
-        <is>
-          <t>資訊單位主管應定期取得重要應用系統之特權帳號及權限清單，覆核帳號擁有者、帳號用途、管理角色、權限範圍、使用狀態及保留必要性；如發現帳號歸屬不明、權限過大或已無使用需求，應即時調整權限或停用帳號，並留存覆核及處理紀錄。</t>
+      <c r="J26" s="61" t="inlineStr">
+        <is>
+          <t>資訊單位主管應定期取得重要應用系統特權帳號及權限清單，覆核擁有者、用途、角色、權限範圍、使用狀態及保留必要性；異常時應調整或停用，並留存覆核及處理紀錄。</t>
         </is>
       </c>
       <c r="K26" s="62" t="inlineStr">
@@ -3622,7 +3649,7 @@
       </c>
       <c r="N26" s="60" t="inlineStr">
         <is>
-          <t>按公司政策"XXX"，針對績效考績系統，原則上為IT人員負責。</t>
+          <t>應用系統特權帳號定期覆核機制未提及。</t>
         </is>
       </c>
       <c r="O26" s="61" t="inlineStr">
@@ -3660,9 +3687,9 @@
           <t>特權存取紀錄覆核</t>
         </is>
       </c>
-      <c r="E27" s="58" t="inlineStr">
-        <is>
-          <t>應用系統特權帳號之異常存取活動未被及時發現及處理</t>
+      <c r="E27" s="61" t="inlineStr">
+        <is>
+          <t>應用系統特權帳號異常存取活動未被及時發現及處理</t>
         </is>
       </c>
       <c r="F27" s="58" t="inlineStr">
@@ -3685,9 +3712,9 @@
           <t>EC-104-04</t>
         </is>
       </c>
-      <c r="J27" s="58" t="inlineStr">
-        <is>
-          <t>資訊單位主管應定期覆核應用系統之特權帳號存取紀錄；若有異常情形，應查明原因並即時處置。</t>
+      <c r="J27" s="61" t="inlineStr">
+        <is>
+          <t>資訊單位主管應定期覆核應用系統特權帳號存取紀錄；異常時應查明原因並即時處置。</t>
         </is>
       </c>
       <c r="K27" s="62" t="inlineStr">
@@ -3707,7 +3734,7 @@
       </c>
       <c r="N27" s="60" t="inlineStr">
         <is>
-          <t>按公司政策"XXX"，針對績效考績系統，原則上為IT人員負責。</t>
+          <t>應用系統特權帳號存取紀錄覆核機制未提及。</t>
         </is>
       </c>
       <c r="O27" s="61" t="inlineStr">
@@ -3745,9 +3772,9 @@
           <t>特權帳號覆核</t>
         </is>
       </c>
-      <c r="E28" s="58" t="inlineStr">
-        <is>
-          <t>正式作業主機之作業系統特權帳號及管理權限遭歸屬不明或已無使用需求之帳號不當使用，或持續保有逾越主機維運需求之權限</t>
+      <c r="E28" s="61" t="inlineStr">
+        <is>
+          <t>作業系統特權帳號歸屬不明、已無需求或權限逾越主機維運需要</t>
         </is>
       </c>
       <c r="F28" s="58" t="inlineStr">
@@ -3770,9 +3797,9 @@
           <t>EC-104-05</t>
         </is>
       </c>
-      <c r="J28" s="58" t="inlineStr">
-        <is>
-          <t>資訊單位主管應定期取得正式作業主機之作業系統特權帳號及管理群組清單，覆核 Administrator、root、sudo、Domain Admins 或其他系統管理權限之帳號擁有者、用途、權限範圍、使用狀態及保留必要性；如有異常，應調整權限或停用帳號，並留存覆核及處理紀錄。</t>
+      <c r="J28" s="61" t="inlineStr">
+        <is>
+          <t>資訊單位主管應定期取得正式作業主機之作業系統特權帳號及管理群組清單，覆核擁有者、用途、權限範圍、使用狀態及保留必要性；異常時應調整或停用，並留存紀錄。</t>
         </is>
       </c>
       <c r="K28" s="62" t="inlineStr">
@@ -3792,7 +3819,7 @@
       </c>
       <c r="N28" s="60" t="inlineStr">
         <is>
-          <t>按公司政策"XXX"，針對績效考績系統，原則上為IT人員負責。</t>
+          <t>作業系統特權帳號定期覆核機制未提及。</t>
         </is>
       </c>
       <c r="O28" s="61" t="inlineStr">
@@ -3830,9 +3857,9 @@
           <t>特權存取紀錄覆核</t>
         </is>
       </c>
-      <c r="E29" s="56" t="inlineStr">
-        <is>
-          <t>作業系統特權帳號之異常存取活動未被及時發現及處理</t>
+      <c r="E29" s="61" t="inlineStr">
+        <is>
+          <t>作業系統特權帳號異常存取活動未被及時發現及處理</t>
         </is>
       </c>
       <c r="F29" s="54" t="inlineStr">
@@ -3855,9 +3882,9 @@
           <t>EC-104-06</t>
         </is>
       </c>
-      <c r="J29" s="56" t="inlineStr">
-        <is>
-          <t>資訊單位主管應定期覆核作業系統之特權帳號存取紀錄；若有異常情形，應查明原因並即時處置。</t>
+      <c r="J29" s="61" t="inlineStr">
+        <is>
+          <t>資訊單位主管應定期覆核作業系統特權帳號存取紀錄；異常時應查明原因並即時處置。</t>
         </is>
       </c>
       <c r="K29" s="55" t="inlineStr">
@@ -3875,9 +3902,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N29" s="63" t="inlineStr">
-        <is>
-          <t>未留下存取紀錄之log，控管方式為權限設定。</t>
+      <c r="N29" s="60" t="inlineStr">
+        <is>
+          <t>未留存作業系統特權帳號存取紀錄，目前僅以權限設定控管。</t>
         </is>
       </c>
       <c r="O29" s="56" t="inlineStr">
@@ -3910,9 +3937,9 @@
           <t>程式及資料之存取控制作業</t>
         </is>
       </c>
-      <c r="D30" s="56" t="inlineStr">
-        <is>
-          <t>資料庫特權存取 / 制度與程序</t>
+      <c r="D30" s="61" t="inlineStr">
+        <is>
+          <t>資料庫特權存取／制度與程序</t>
         </is>
       </c>
       <c r="E30" s="62" t="inlineStr">
@@ -3960,14 +3987,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N30" s="63" t="inlineStr">
-        <is>
-          <t>1.資料庫變更：原則上不允許，惟曾因組織調整而執行的大批量部門編號異動，係由資訊人員直接在後台執行，該作業並無正式書面核准紀錄。
-2.稽核軌跡：前 Office 365 具備內建監控功能，但核心系統如 ERP 則明確表示目前無存取監控機制，目前亦無詳細的變更日誌（Change Log）或稽核軌跡可供查核。
-3.權限設定：目前同仁均配發獨立帳號與密碼，存取權限係依據人事單位的組織架構圖進行設定與鎖定。
-4.經應用程式修改資料庫：未提及
-5.資料庫備份：系統具備每日凌晨自動備份機制，並留存 90 個歷史版本。
-6.迅速取得備援資料庫：未提及</t>
+      <c r="N30" s="60" t="inlineStr">
+        <is>
+          <t>資料庫直接異動原則上不允許；曾由資訊人員於後台執行大批量部門編號異動，無書面核准紀錄。ERP 等核心系統無存取監控及變更日誌。</t>
         </is>
       </c>
       <c r="O30" s="58" t="inlineStr">
@@ -4009,9 +4031,9 @@
           <t>特權帳號覆核</t>
         </is>
       </c>
-      <c r="E31" s="58" t="inlineStr">
-        <is>
-          <t>重要資料庫之特權帳號、角色及系統權限遭歸屬不明或已無使用需求之帳號不當使用，或持續保有逾越資料庫維運需求之存取權限</t>
+      <c r="E31" s="61" t="inlineStr">
+        <is>
+          <t>資料庫特權帳號、角色或權限歸屬不明、已無需求或逾越維運需要</t>
         </is>
       </c>
       <c r="F31" s="58" t="inlineStr">
@@ -4034,9 +4056,9 @@
           <t>EC-104-08</t>
         </is>
       </c>
-      <c r="J31" s="58" t="inlineStr">
-        <is>
-          <t>資訊單位主管應定期取得重要資料庫之特權帳號、角色及系統權限清單，覆核資料庫管理員、系統服務帳號及其他高權限帳號之擁有者、用途、存取範圍、使用狀態及保留必要性；如有異常，應調整權限或停用帳號，並留存覆核及處理紀錄。</t>
+      <c r="J31" s="61" t="inlineStr">
+        <is>
+          <t>資訊單位主管應定期取得重要資料庫特權帳號、角色及系統權限清單並覆核；異常時應調整或停用，並留存紀錄。</t>
         </is>
       </c>
       <c r="K31" s="62" t="inlineStr">
@@ -4056,7 +4078,7 @@
       </c>
       <c r="N31" s="60" t="inlineStr">
         <is>
-          <t>按公司政策"XXX"，針對績效考績系統，原則上為IT人員負責。</t>
+          <t>資料庫特權帳號定期覆核機制未提及。</t>
         </is>
       </c>
       <c r="O31" s="61" t="inlineStr">
@@ -4094,9 +4116,9 @@
           <t>特權存取紀錄覆核</t>
         </is>
       </c>
-      <c r="E32" s="56" t="inlineStr">
-        <is>
-          <t>資料庫特權帳號之異常存取活動未被及時發現及處理</t>
+      <c r="E32" s="61" t="inlineStr">
+        <is>
+          <t>資料庫特權帳號異常存取活動未被及時發現及處理</t>
         </is>
       </c>
       <c r="F32" s="54" t="inlineStr">
@@ -4119,9 +4141,9 @@
           <t>EC-104-09</t>
         </is>
       </c>
-      <c r="J32" s="56" t="inlineStr">
-        <is>
-          <t>資訊單位主管應定期覆核資料庫之特權帳號存取紀錄；若有異常情形，應查明原因並即時處置。</t>
+      <c r="J32" s="61" t="inlineStr">
+        <is>
+          <t>資訊單位主管應定期覆核資料庫特權帳號存取紀錄；異常時應查明原因並即時處置。</t>
         </is>
       </c>
       <c r="K32" s="55" t="inlineStr">
@@ -4139,9 +4161,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N32" s="63" t="inlineStr">
-        <is>
-          <t>未留下存取紀錄之log，控管方式為權限設定。</t>
+      <c r="N32" s="60" t="inlineStr">
+        <is>
+          <t>未留存資料庫特權帳號存取紀錄，目前僅以權限設定控管。</t>
         </is>
       </c>
       <c r="O32" s="56" t="inlineStr">
@@ -4179,9 +4201,9 @@
           <t>特權帳號覆核</t>
         </is>
       </c>
-      <c r="E33" s="58" t="inlineStr">
-        <is>
-          <t>重要網路相關系統之特權帳號及管理權限遭歸屬不明或已無使用需求之帳號不當使用，或持續保有逾越網路維運需求之權限</t>
+      <c r="E33" s="61" t="inlineStr">
+        <is>
+          <t>網路相關系統特權帳號歸屬不明、已無需求或權限逾越維運需要</t>
         </is>
       </c>
       <c r="F33" s="58" t="inlineStr">
@@ -4204,9 +4226,9 @@
           <t>EC-104-10</t>
         </is>
       </c>
-      <c r="J33" s="58" t="inlineStr">
-        <is>
-          <t>資訊單位主管應定期取得防火牆、交換器、路由器、VPN 及其他重要網路相關系統之特權帳號及權限清單，覆核帳號擁有者、用途、管理權限、使用狀態及保留必要性；如有異常，應調整權限或停用帳號，並留存覆核及處理紀錄。</t>
+      <c r="J33" s="61" t="inlineStr">
+        <is>
+          <t>資訊單位主管應定期取得防火牆、交換器、路由器、VPN 等網路系統特權帳號及權限清單並覆核；異常時應調整或停用，並留存紀錄。</t>
         </is>
       </c>
       <c r="K33" s="62" t="inlineStr">
@@ -4226,7 +4248,7 @@
       </c>
       <c r="N33" s="60" t="inlineStr">
         <is>
-          <t>按公司政策"XXX"，針對績效考績系統，原則上為IT人員負責。</t>
+          <t>網路系統特權帳號定期覆核機制未提及。</t>
         </is>
       </c>
       <c r="O33" s="61" t="inlineStr">
@@ -4264,9 +4286,9 @@
           <t>特權存取紀錄覆核</t>
         </is>
       </c>
-      <c r="E34" s="56" t="inlineStr">
-        <is>
-          <t>網路相關系統特權帳號之異常存取活動未被及時發現及處理</t>
+      <c r="E34" s="61" t="inlineStr">
+        <is>
+          <t>網路相關系統特權帳號異常存取活動未被及時發現及處理</t>
         </is>
       </c>
       <c r="F34" s="54" t="inlineStr">
@@ -4289,9 +4311,9 @@
           <t>EC-104-11</t>
         </is>
       </c>
-      <c r="J34" s="56" t="inlineStr">
-        <is>
-          <t>資訊單位主管應定期覆核網路相關系統之特權帳號存取紀錄；若有異常情形，應查明原因並即時處置。</t>
+      <c r="J34" s="61" t="inlineStr">
+        <is>
+          <t>資訊單位主管應定期覆核網路相關系統特權帳號存取紀錄；異常時應查明原因並即時處置。</t>
         </is>
       </c>
       <c r="K34" s="55" t="inlineStr">
@@ -4309,9 +4331,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N34" s="63" t="inlineStr">
-        <is>
-          <t>未留下存取紀錄之log，控管方式為權限設定。</t>
+      <c r="N34" s="60" t="inlineStr">
+        <is>
+          <t>未留存網路系統特權帳號存取紀錄，目前僅以權限設定控管。</t>
         </is>
       </c>
       <c r="O34" s="56" t="inlineStr">
@@ -4349,9 +4371,9 @@
           <t>共用帳號</t>
         </is>
       </c>
-      <c r="E35" s="56" t="inlineStr">
-        <is>
-          <t>系統操作因無法追溯至實際執行人員，而在發生未經授權存取、資料不當異動或異常行為時難以究責</t>
+      <c r="E35" s="61" t="inlineStr">
+        <is>
+          <t>系統操作無法追溯至實際執行人員，異常行為難以究責</t>
         </is>
       </c>
       <c r="F35" s="54" t="inlineStr">
@@ -4394,9 +4416,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N35" s="67" t="inlineStr">
-        <is>
-          <t>管理員（特權）帳號，目前由資訊主管與 IT 人員分別持有相關管理權限，其中 Office 365 帳號由主管控管，而其餘系統管理則在 IT 人員手中。</t>
+      <c r="N35" s="76" t="inlineStr">
+        <is>
+          <t>一般同仁配發個人帳號。特權管理權限由資訊單位主管與資訊人員分別持有：Office 365 由主管控管，其餘系統管理多由資訊人員負責。</t>
         </is>
       </c>
       <c r="O35" s="66" t="n"/>
@@ -4430,9 +4452,9 @@
           <t>使用者帳號管理</t>
         </is>
       </c>
-      <c r="E36" s="56" t="inlineStr">
-        <is>
-          <t>使用者系統帳號及存取權限因未隨晉升、調職或離職情形即時調整，而遭離職人員或職務已變更人員未經授權使用</t>
+      <c r="E36" s="61" t="inlineStr">
+        <is>
+          <t>帳號及權限未隨入職、調職或離職即時調整，遭無權人員使用</t>
         </is>
       </c>
       <c r="F36" s="54" t="inlineStr">
@@ -4455,9 +4477,9 @@
           <t>EC-104-13</t>
         </is>
       </c>
-      <c r="J36" s="56" t="inlineStr">
-        <is>
-          <t>員工晉升、調職或離職時，應有適當之系統帳戶新增、修改及刪除程序，以便依其新狀況調整資訊資源之授權。</t>
+      <c r="J36" s="61" t="inlineStr">
+        <is>
+          <t>員工入職、調職或離職時，應依程序新增、修改或刪除系統帳號及權限，使授權與職務相符。</t>
         </is>
       </c>
       <c r="K36" s="55" t="inlineStr">
@@ -4475,9 +4497,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N36" s="68" t="inlineStr">
-        <is>
-          <t>目前公司針對員工入職、調職或離職之帳號與權限異動，係透過電子簽核系統提出申請並留存軌跡，且系統授權係依據人事單位維護之組織架構圖進行對應設定。</t>
+      <c r="N36" s="60" t="inlineStr">
+        <is>
+          <t>入職、調職或離職之帳號與權限異動透過電子簽核提出申請並留存軌跡；授權多依人事單位組織架構圖設定。</t>
         </is>
       </c>
       <c r="O36" s="56" t="inlineStr">
@@ -4511,14 +4533,14 @@
           <t>程式及資料之存取控制作業</t>
         </is>
       </c>
-      <c r="D37" s="56" t="inlineStr">
-        <is>
-          <t>密碼管理 / 制度與程序</t>
-        </is>
-      </c>
-      <c r="E37" s="56" t="inlineStr">
-        <is>
-          <t>重要系統帳號易遭密碼破解或帳號冒用，使未經授權人員得以存取系統及相關資料</t>
+      <c r="D37" s="61" t="inlineStr">
+        <is>
+          <t>密碼管理／制度與程序</t>
+        </is>
+      </c>
+      <c r="E37" s="61" t="inlineStr">
+        <is>
+          <t>重要系統帳號易遭密碼破解或冒用，使未經授權人員存取系統及資料</t>
         </is>
       </c>
       <c r="F37" s="58" t="inlineStr">
@@ -4541,9 +4563,9 @@
           <t>EC-104-14</t>
         </is>
       </c>
-      <c r="J37" s="56" t="inlineStr">
-        <is>
-          <t>重要系統皆應設定相關密碼規則（包含：密碼長度、密碼強度、密碼定期更換、可接受之密碼錯誤次數、重覆密碼控制）。</t>
+      <c r="J37" s="61" t="inlineStr">
+        <is>
+          <t>重要系統應設定密碼規則，包括長度、強度、定期更換、錯誤次數上限及重複密碼控制。</t>
         </is>
       </c>
       <c r="K37" s="55" t="inlineStr">
@@ -4561,9 +4583,9 @@
           <t>持續</t>
         </is>
       </c>
-      <c r="N37" s="68" t="inlineStr">
-        <is>
-          <t>公司尚無密碼政策，僅Office 365使用該系統既定規則定期更換密碼。</t>
+      <c r="N37" s="60" t="inlineStr">
+        <is>
+          <t>公司尚無統一密碼政策；僅 Office 365 依系統既定規則定期更換密碼。</t>
         </is>
       </c>
       <c r="O37" s="56" t="inlineStr">
@@ -4601,9 +4623,9 @@
           <t>密碼管理</t>
         </is>
       </c>
-      <c r="E38" s="56" t="inlineStr">
-        <is>
-          <t>使用者帳號遭冒用及機密資料被未經授權存取或外洩</t>
+      <c r="E38" s="61" t="inlineStr">
+        <is>
+          <t>使用者持續使用初始密碼，致帳號遭冒用或資料外洩</t>
         </is>
       </c>
       <c r="F38" s="58" t="inlineStr">
@@ -4626,9 +4648,9 @@
           <t>EC-104-15</t>
         </is>
       </c>
-      <c r="J38" s="56" t="inlineStr">
-        <is>
-          <t>一般使用者帳號建立或密碼重置後，應由使用者於首次登入時變更初始密碼；初始密碼不得由不同使用者共同使用。</t>
+      <c r="J38" s="61" t="inlineStr">
+        <is>
+          <t>一般使用者帳號建立或密碼重置後，應於首次登入變更初始密碼；初始密碼不得由不同使用者共用。</t>
         </is>
       </c>
       <c r="K38" s="55" t="inlineStr">
@@ -4682,9 +4704,9 @@
           <t>使用者權限覆核</t>
         </is>
       </c>
-      <c r="E39" s="56" t="inlineStr">
-        <is>
-          <t>使用者系統存取權限因未經定期覆核及即時調整，而遭使用者逾越現行職務範圍存取或使用系統資源</t>
+      <c r="E39" s="61" t="inlineStr">
+        <is>
+          <t>使用者權限未經定期覆核及調整，致逾越現行職務範圍存取系統</t>
         </is>
       </c>
       <c r="F39" s="54" t="inlineStr">
@@ -4697,9 +4719,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="H39" s="58" t="inlineStr">
-        <is>
-          <t>應用系統權限帳號皆與其擁有者工作職責相符</t>
+      <c r="H39" s="61" t="inlineStr">
+        <is>
+          <t>應用系統使用者權限與其工作職責相符</t>
         </is>
       </c>
       <c r="I39" s="59" t="inlineStr">
@@ -4707,9 +4729,9 @@
           <t>EC-104-16</t>
         </is>
       </c>
-      <c r="J39" s="56" t="inlineStr">
-        <is>
-          <t>使用單位主管應定期取得並覆核使用者權限清單；若有不適當者，應即時申請移除該帳號權限或停權。</t>
+      <c r="J39" s="61" t="inlineStr">
+        <is>
+          <t>使用單位主管應定期取得並覆核使用者權限清單；不適當者應即時申請移除或停權。</t>
         </is>
       </c>
       <c r="K39" s="55" t="inlineStr">
@@ -4763,9 +4785,9 @@
           <t>使用者存取紀錄覆核</t>
         </is>
       </c>
-      <c r="E40" s="56" t="inlineStr">
-        <is>
-          <t>未經授權登入、逾越職務範圍存取或大量資料下載等異常行為未被及時發現及處理</t>
+      <c r="E40" s="61" t="inlineStr">
+        <is>
+          <t>未經授權登入、逾權存取或大量下載等異常行為未被及時發現及處理</t>
         </is>
       </c>
       <c r="F40" s="54" t="inlineStr">
@@ -4788,9 +4810,9 @@
           <t>EC-104-17</t>
         </is>
       </c>
-      <c r="J40" s="56" t="inlineStr">
-        <is>
-          <t>應用系統管理者應定期產出重要或敏感系統之異常使用者存取紀錄，包括非正常時段登入、重複登入失敗、異常來源登入、大量資料查詢或下載及逾越職務範圍之存取活動；發現異常時，應提交系統擁有者或使用單位主管覆核其業務合理性，並留存處理結果。</t>
+      <c r="J40" s="61" t="inlineStr">
+        <is>
+          <t>應用系統管理者應定期產出重要或敏感系統之異常存取紀錄（含非正常時段登入、重複登入失敗、異常來源、大量查詢或下載及逾權存取），提交系統擁有者或使用單位主管覆核合理性，並留存處理結果。</t>
         </is>
       </c>
       <c r="K40" s="55" t="inlineStr">
@@ -4808,9 +4830,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N40" s="68" t="inlineStr">
-        <is>
-          <t>未留下存取紀錄之log，控管方式為權限設定。</t>
+      <c r="N40" s="60" t="inlineStr">
+        <is>
+          <t>未留存使用者存取紀錄，目前僅以權限設定控管。</t>
         </is>
       </c>
       <c r="O40" s="56" t="inlineStr">
@@ -4848,9 +4870,9 @@
           <t>資料輸入控制</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>不完整資料輸入系統，影響資料品質及後續作業結果</t>
+      <c r="E41" s="61" t="inlineStr">
+        <is>
+          <t>不完整資料輸入系統，影響資料品質及後續作業</t>
         </is>
       </c>
       <c r="F41" s="1" t="inlineStr">
@@ -4925,9 +4947,9 @@
           <t>資料輸入控制</t>
         </is>
       </c>
-      <c r="E42" s="3" t="inlineStr">
-        <is>
-          <t>錯誤或不合理資料輸入系統，影響資料品質及後續作業結果</t>
+      <c r="E42" s="61" t="inlineStr">
+        <is>
+          <t>錯誤或不合理資料輸入系統，影響資料品質及後續作業</t>
         </is>
       </c>
       <c r="F42" s="1" t="inlineStr">
@@ -5002,9 +5024,9 @@
           <t>資料輸入控制</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>重複資料輸入系統，影響資料品質及後續作業結果</t>
+      <c r="E43" s="61" t="inlineStr">
+        <is>
+          <t>重複資料輸入系統，影響資料品質及後續作業</t>
         </is>
       </c>
       <c r="F43" s="1" t="inlineStr">
@@ -5017,9 +5039,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>系統內資料數據完整且妥善整理</t>
+      <c r="H43" s="61" t="inlineStr">
+        <is>
+          <t>系統資料避免重複建立或輸入</t>
         </is>
       </c>
       <c r="I43" s="9" t="inlineStr">
@@ -5074,14 +5096,14 @@
           <t>資料輸出入控制作業</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>資料存取控制 / 資料輸出控制</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>保管資料因未經權責主管核准即遭撈取移交，而被非必要人員取得或不當使用</t>
+      <c r="D44" s="61" t="inlineStr">
+        <is>
+          <t>資料存取控制／資料輸出控制</t>
+        </is>
+      </c>
+      <c r="E44" s="61" t="inlineStr">
+        <is>
+          <t>保管資料未經權責主管核准即遭撈取移交，被非必要人員取得或不當使用</t>
         </is>
       </c>
       <c r="F44" s="1" t="inlineStr">
@@ -5124,9 +5146,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N44" s="52" t="inlineStr">
-        <is>
-          <t>目前公司針對主要系統（如 Office 365、NAS、FTP、ERP）之帳號新增與資料存取權限，已要求同仁透過電子簽核系統（EasyFlow）填寫表單提出申請，並經由相關權責主管核准後留存軌跡。針對特定的敏感資料（如營業秘密），亦設有專門的申請程序，需經由法務部審核並記錄存取人員名單。</t>
+      <c r="N44" s="60" t="inlineStr">
+        <is>
+          <t>主要系統（Office 365、NAS、FTP、ERP）帳號新增與資料存取權限，須經電子簽核（EasyFlow）申請並由權責主管核准。營業秘密等機敏資料另經法務審核並記錄存取人員。</t>
         </is>
       </c>
       <c r="O44" s="3" t="n"/>
@@ -5160,9 +5182,9 @@
           <t>機密資料保護</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>公司特定單位機密性或敏感性資料遭單位外人員取得或洩漏</t>
+      <c r="E45" s="61" t="inlineStr">
+        <is>
+          <t>單位機密或敏感性資料遭單位外人員取得或洩漏</t>
         </is>
       </c>
       <c r="F45" s="1" t="inlineStr">
@@ -5205,9 +5227,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N45" s="50" t="inlineStr">
-        <is>
-          <t>欲拜訪、存取機敏資料如營業秘密，需透過電子簽核系統進行申請。</t>
+      <c r="N45" s="60" t="inlineStr">
+        <is>
+          <t>調閱或存取營業秘密等機敏資料，須經電子簽核申請。</t>
         </is>
       </c>
       <c r="O45" s="3" t="n"/>
@@ -5236,14 +5258,14 @@
           <t>資料輸出入控制作業</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>個人資料保護 / 資料輸出控制</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr">
-        <is>
-          <t>公司或員工違反個人資料保護相關法規</t>
+      <c r="D46" s="61" t="inlineStr">
+        <is>
+          <t>個人資料保護／資料輸出控制</t>
+        </is>
+      </c>
+      <c r="E46" s="61" t="inlineStr">
+        <is>
+          <t>個人資料之蒐集、處理或利用違反公司規定或相關法規</t>
         </is>
       </c>
       <c r="F46" s="1" t="inlineStr">
@@ -5286,9 +5308,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N46" s="52" t="inlineStr">
-        <is>
-          <t>欲拜訪、存取機敏資料如營業秘密，需透過電子簽核系統進行申請。</t>
+      <c r="N46" s="60" t="inlineStr">
+        <is>
+          <t>調閱或存取營業秘密等機敏資料，須經電子簽核申請；個人資料專責申請流程待確認。</t>
         </is>
       </c>
       <c r="O46" s="3" t="n"/>
@@ -5322,9 +5344,9 @@
           <t>資料庫資料處理</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>資料庫資料遭直接異動，而發生未經授權或錯誤之新增、修改、刪除及操作無法追溯</t>
+      <c r="E47" s="61" t="inlineStr">
+        <is>
+          <t>資料庫資料遭直接異動，發生未經授權或錯誤之增刪修，且無法追溯</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -5367,14 +5389,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N47" s="53" t="inlineStr">
-        <is>
-          <t>1.資料庫變更：原則上不允許，惟曾因組織調整而執行的大批量部門編號異動，係由資訊人員直接在後台執行，該作業並無正式書面核准紀錄。
-2.稽核軌跡：前 Office 365 具備內建監控功能，但核心系統如 ERP 則明確表示目前無存取監控機制，目前亦無詳細的變更日誌（Change Log）或稽核軌跡可供查核。
-3.權限設定：目前同仁均配發獨立帳號與密碼，存取權限係依據人事單位的組織架構圖進行設定與鎖定。
-4.經應用程式修改資料庫：未提及
-5.資料庫備份：系統具備每日凌晨自動備份機制，並留存 90 個歷史版本。
-6.迅速取得備援資料庫：未提及</t>
+      <c r="N47" s="60" t="inlineStr">
+        <is>
+          <t>資料庫直接異動原則上不允許；曾由資訊人員於後台執行大批量部門編號異動，無書面核准紀錄。ERP 等核心系統無存取監控及變更日誌。</t>
         </is>
       </c>
       <c r="O47" s="2" t="inlineStr">
@@ -5408,14 +5425,14 @@
           <t>資料處理之控制作業</t>
         </is>
       </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>系統工作排程 / 排程授權管理</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>系統工作排程發生資料處理錯誤、排程遺漏或非預期作業中斷</t>
+      <c r="D48" s="61" t="inlineStr">
+        <is>
+          <t>系統工作排程／排程授權管理</t>
+        </is>
+      </c>
+      <c r="E48" s="61" t="inlineStr">
+        <is>
+          <t>系統工作排程發生處理錯誤、遺漏或非預期中斷</t>
         </is>
       </c>
       <c r="F48" s="1" t="inlineStr">
@@ -5458,9 +5475,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N48" s="50" t="inlineStr">
-        <is>
-          <t>目前公司無跑批作業</t>
+      <c r="N48" s="60" t="inlineStr">
+        <is>
+          <t>目前無批次作業</t>
         </is>
       </c>
       <c r="O48" s="50" t="inlineStr">
@@ -5493,14 +5510,14 @@
           <t>資料處理之控制作業</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>系統工作排程 / 排程定期覆核</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>系統工作排程因設定錯誤、執行異常或已無使用需求，而影響資料處理及系統作業之正常執行</t>
+      <c r="D49" s="61" t="inlineStr">
+        <is>
+          <t>系統工作排程／排程定期覆核</t>
+        </is>
+      </c>
+      <c r="E49" s="61" t="inlineStr">
+        <is>
+          <t>系統工作排程設定錯誤、執行異常或已無需求，影響資料處理及系統作業</t>
         </is>
       </c>
       <c r="F49" s="1" t="inlineStr">
@@ -5543,9 +5560,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N49" s="50" t="inlineStr">
-        <is>
-          <t>目前公司無跑批作業</t>
+      <c r="N49" s="60" t="inlineStr">
+        <is>
+          <t>目前無批次作業</t>
         </is>
       </c>
       <c r="O49" s="50" t="inlineStr">
@@ -5578,14 +5595,14 @@
           <t>資料處理之控制作業</t>
         </is>
       </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>系統工作排程 / 排程監控</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr">
-        <is>
-          <t>系統工作排程因執行失敗、延遲或其他例外情形，而使資料處理不完整、不正確或未依預定時程完成</t>
+      <c r="D50" s="61" t="inlineStr">
+        <is>
+          <t>系統工作排程／排程監控</t>
+        </is>
+      </c>
+      <c r="E50" s="61" t="inlineStr">
+        <is>
+          <t>系統工作排程執行失敗、延遲或其他例外，致資料處理不完整、不正確或未依時程完成</t>
         </is>
       </c>
       <c r="F50" s="1" t="inlineStr">
@@ -5628,9 +5645,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N50" s="50" t="inlineStr">
-        <is>
-          <t>目前公司無跑批作業</t>
+      <c r="N50" s="60" t="inlineStr">
+        <is>
+          <t>目前無批次作業</t>
         </is>
       </c>
       <c r="O50" s="50" t="inlineStr">
@@ -5668,9 +5685,9 @@
           <t>系統組態異動紀錄</t>
         </is>
       </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>正式作業環境之系統參數、平台設定或系統組態因錯誤或與核准需求不一致之異動，而使系統功能異常、資料處理錯誤或服務中斷</t>
+      <c r="E51" s="61" t="inlineStr">
+        <is>
+          <t>正式作業環境之系統參數、平台或組態異動錯誤或與核准不符，致功能異常、資料錯誤或服務中斷</t>
         </is>
       </c>
       <c r="F51" s="1" t="inlineStr">
@@ -5713,9 +5730,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N51" s="52" t="inlineStr">
-        <is>
-          <t>績效考績系統更新過板後留下100個程式碼舊版本。</t>
+      <c r="N51" s="60" t="inlineStr">
+        <is>
+          <t>績效考核系統過版後保留約 100 個程式舊版本；系統參數及組態異動之完整前後比對紀錄待確認。</t>
         </is>
       </c>
       <c r="O51" s="3" t="n"/>
@@ -5749,9 +5766,9 @@
           <t>系統組態異常回復</t>
         </is>
       </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>系統參數或組態設定異常因未及時回復，而影響系統功能及正常運行</t>
+      <c r="E52" s="61" t="inlineStr">
+        <is>
+          <t>系統參數或組態異常未及時回復，影響系統功能及正常運行</t>
         </is>
       </c>
       <c r="F52" s="1" t="inlineStr">
@@ -5830,9 +5847,9 @@
           <t>作業系統變更管理</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>作業系統因未經授權或不當變更而中斷、功能異常或資安漏洞，破壞正式環境穩定性及資訊安全</t>
+      <c r="E53" s="61" t="inlineStr">
+        <is>
+          <t>作業系統未經授權或不當變更，致中斷、功能異常或資安漏洞</t>
         </is>
       </c>
       <c r="F53" s="1" t="inlineStr">
@@ -5875,9 +5892,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N53" s="52" t="inlineStr">
-        <is>
-          <t>目前大多透過會議口頭討論執行，並無正式的書面核准紀錄。</t>
+      <c r="N53" s="60" t="inlineStr">
+        <is>
+          <t>多以會議口頭討論執行，無書面核准紀錄。</t>
         </is>
       </c>
       <c r="O53" s="3" t="inlineStr">
@@ -5910,14 +5927,14 @@
           <t>檔案及設備之安全控制作業</t>
         </is>
       </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>軟硬體存取控制 / 密碼政策</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>公司電腦軟硬體所儲存或處理之機密或敏感資料遭未經授權存取、使用或揭露</t>
+      <c r="D54" s="61" t="inlineStr">
+        <is>
+          <t>軟硬體存取控制／密碼政策</t>
+        </is>
+      </c>
+      <c r="E54" s="61" t="inlineStr">
+        <is>
+          <t>電腦軟硬體所儲存或處理之機密或敏感資料遭未經授權存取、使用或揭露</t>
         </is>
       </c>
       <c r="F54" s="1" t="inlineStr">
@@ -6000,9 +6017,9 @@
           <t>機房進出管制</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t>未經授權人員進出機房致重要資料毀損或洩漏</t>
+      <c r="E55" s="61" t="inlineStr">
+        <is>
+          <t>未經授權人員進出機房，致重要資料毀損或洩漏</t>
         </is>
       </c>
       <c r="F55" s="1" t="inlineStr">
@@ -6045,9 +6062,9 @@
           <t>持續</t>
         </is>
       </c>
-      <c r="N55" s="52" t="inlineStr">
-        <is>
-          <t>機房設有進入權限控管（門禁管制），且具備相關的門禁進出紀錄。</t>
+      <c r="N55" s="60" t="inlineStr">
+        <is>
+          <t>機房設有門禁管制，並留存進出紀錄。</t>
         </is>
       </c>
       <c r="O55" s="3" t="n"/>
@@ -6081,9 +6098,9 @@
           <t>機房進出管制</t>
         </is>
       </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>未經授權人員進出機房致重要資料毀損或洩漏</t>
+      <c r="E56" s="61" t="inlineStr">
+        <is>
+          <t>未經授權人員進出機房，致重要資料毀損或洩漏</t>
         </is>
       </c>
       <c r="F56" s="1" t="inlineStr">
@@ -6126,9 +6143,9 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="N56" s="50" t="inlineStr">
-        <is>
-          <t>TBC：機房進出人員須向資訊主管事前申請…</t>
+      <c r="N56" s="60" t="inlineStr">
+        <is>
+          <t>機房進出須向資訊單位主管事前申請（細節待確認）。</t>
         </is>
       </c>
       <c r="O56" s="3" t="n"/>
@@ -6162,9 +6179,9 @@
           <t>機房進出管制</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr">
-        <is>
-          <t>未經授權人員進出機房致重要資料毀損或洩漏</t>
+      <c r="E57" s="61" t="inlineStr">
+        <is>
+          <t>機房進出異常未被定期覆核及處理</t>
         </is>
       </c>
       <c r="F57" s="1" t="inlineStr">
@@ -6243,9 +6260,9 @@
           <t>設備之安全控制</t>
         </is>
       </c>
-      <c r="E58" s="3" t="inlineStr">
-        <is>
-          <t>機房因硬體設備老舊過期致無法因應重大事故而毀損停擺</t>
+      <c r="E58" s="61" t="inlineStr">
+        <is>
+          <t>機房硬體或消防設施欠缺維護，重大事故時無法運作</t>
         </is>
       </c>
       <c r="F58" s="1" t="inlineStr">
@@ -6288,14 +6305,9 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="N58" s="50" t="inlineStr">
-        <is>
-          <t>1. 未提及
-2. 未提及
-3. 無
-4. 未提及
-5. 未提及
-6. 委外廠商於合約簽署NDA</t>
+      <c r="N58" s="60" t="inlineStr">
+        <is>
+          <t>電腦設備及周邊定期維修檢查未提及；委外廠商合約有簽署 NDA。</t>
         </is>
       </c>
       <c r="O58" s="7" t="inlineStr">
@@ -6337,9 +6349,9 @@
           <t>備援設備維護</t>
         </is>
       </c>
-      <c r="E59" s="3" t="inlineStr">
-        <is>
-          <t>重要資訊在設備故障或電力異常時發生系統中斷或資料流失</t>
+      <c r="E59" s="61" t="inlineStr">
+        <is>
+          <t>設備故障或電力異常時，發生系統中斷或資料流失</t>
         </is>
       </c>
       <c r="F59" s="1" t="inlineStr">
@@ -6422,9 +6434,9 @@
           <t>儲存媒體管理</t>
         </is>
       </c>
-      <c r="E60" s="3" t="inlineStr">
-        <is>
-          <t>儲存媒體因內容、用途或識別資訊不明，而遭錯誤取用、誤用或不當處置，致其所儲存資料遺失、毀損或外洩</t>
+      <c r="E60" s="61" t="inlineStr">
+        <is>
+          <t>儲存媒體內容、用途或識別不明，遭誤用或不當處置，致資料遺失、毀損或外洩</t>
         </is>
       </c>
       <c r="F60" s="1" t="inlineStr">
@@ -6548,12 +6560,9 @@
         </is>
       </c>
       <c r="M61" s="9" t="n"/>
-      <c r="N61" s="50" t="inlineStr">
-        <is>
-          <t>1.備份機制：目前公司針對主要系統（如 ERP）與重要資料執行每日自動備份（凌晨 3 點執行），且具備 90 個版本之留存機制。備份採用異地同步模式，由台北 NAS 自動同步至新竹 NAS。
-2.專人保管：未提及
-3.防毒軟體管理：未提及
-4.人員訓練：未提及</t>
+      <c r="N61" s="60" t="inlineStr">
+        <is>
+          <t>主要系統（如 ERP）及重要資料每日自動備份（約凌晨 3 時），保留 90 個版本；台北 NAS 異地同步至新竹 NAS。專人保管機制未提及。</t>
         </is>
       </c>
       <c r="O61" s="7" t="inlineStr">
@@ -6586,14 +6595,14 @@
           <t>硬體及系統軟體之購置、使用及維護控制作業</t>
         </is>
       </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>資訊採購 / 制度與程序</t>
-        </is>
-      </c>
-      <c r="E62" s="3" t="inlineStr">
-        <is>
-          <t>資訊類採購因評選標準不明確或不符合資訊安全需求，而取得不符公司需求或安全規範之資訊產品及服務</t>
+      <c r="D62" s="61" t="inlineStr">
+        <is>
+          <t>資訊採購／制度與程序</t>
+        </is>
+      </c>
+      <c r="E62" s="61" t="inlineStr">
+        <is>
+          <t>資訊類採購評選標準不明或不符資安需求，取得不符需求或安全規範之產品及服務</t>
         </is>
       </c>
       <c r="F62" s="1" t="inlineStr">
@@ -6676,9 +6685,9 @@
           <t>資訊採購</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>資訊系統採購不符合公司需求或缺乏成本效益</t>
+      <c r="E63" s="61" t="inlineStr">
+        <is>
+          <t>資訊系統採購不符公司需求或缺乏成本效益</t>
         </is>
       </c>
       <c r="F63" s="1" t="inlineStr">
@@ -6761,9 +6770,9 @@
           <t>無形資產管理</t>
         </is>
       </c>
-      <c r="E64" s="3" t="inlineStr">
-        <is>
-          <t>系統軟體因授權無效、逾期或超出授權範圍使用，而使公司承擔侵權或違約責任</t>
+      <c r="E64" s="61" t="inlineStr">
+        <is>
+          <t>系統軟體授權無效、逾期或超出範圍使用，致侵權或違約</t>
         </is>
       </c>
       <c r="F64" s="1" t="inlineStr">
@@ -6846,9 +6855,9 @@
           <t>資訊資產管理</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>公司資訊資產遭侵占或變賣而難以即時發現</t>
+      <c r="E65" s="61" t="inlineStr">
+        <is>
+          <t>資訊資產遭侵占或變賣而難以即時發現</t>
         </is>
       </c>
       <c r="F65" s="1" t="inlineStr">
@@ -6931,9 +6940,9 @@
           <t>資訊資產移轉</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>公司資訊資產遭侵占或變賣而難以即時發現</t>
+      <c r="E66" s="61" t="inlineStr">
+        <is>
+          <t>資訊資產移動或移轉未經核准，致資產流失或狀態不明</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -7016,9 +7025,9 @@
           <t>資訊資產管理</t>
         </is>
       </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>公司資訊資產遭侵占或變賣而難以即時發現</t>
+      <c r="E67" s="61" t="inlineStr">
+        <is>
+          <t>資訊資產移動或移轉後清冊未更新，致資產狀態不明</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -7051,9 +7060,9 @@
           <t>人工</t>
         </is>
       </c>
-      <c r="L67" s="32" t="inlineStr">
-        <is>
-          <t>偵測系控制</t>
+      <c r="L67" s="59" t="inlineStr">
+        <is>
+          <t>偵測性控制</t>
         </is>
       </c>
       <c r="M67" s="30" t="inlineStr">
@@ -7101,9 +7110,9 @@
           <t>資訊設備維護</t>
         </is>
       </c>
-      <c r="E68" s="3" t="inlineStr">
-        <is>
-          <t>公司電腦硬體因欠缺維護而提早毀損</t>
+      <c r="E68" s="61" t="inlineStr">
+        <is>
+          <t>電腦硬體欠缺維護而提早毀損</t>
         </is>
       </c>
       <c r="F68" s="1" t="inlineStr">
@@ -7146,9 +7155,9 @@
           <t>每年</t>
         </is>
       </c>
-      <c r="N68" s="52" t="inlineStr">
-        <is>
-          <t>外購軟體透過年度合約進行維護。硬體設備未提及</t>
+      <c r="N68" s="60" t="inlineStr">
+        <is>
+          <t>外購軟體依年度合約維護；硬體設備定期維護未提及。</t>
         </is>
       </c>
       <c r="O68" s="3" t="n"/>
@@ -7207,9 +7216,9 @@
           <t>EC-108-08</t>
         </is>
       </c>
-      <c r="J69" s="2" t="inlineStr">
-        <is>
-          <t>使用部門電腦軟硬體申請報修，應提交報修物品並留存申請紀錄，由資訊部門記錄故障原因並評估維修可能性。</t>
+      <c r="J69" s="61" t="inlineStr">
+        <is>
+          <t>使用部門電腦軟硬體申請報修，應提交報修物品並留存申請紀錄，由資訊單位記錄故障原因並評估維修可能性。</t>
         </is>
       </c>
       <c r="K69" s="9" t="inlineStr">
@@ -7227,9 +7236,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N69" s="52" t="inlineStr">
-        <is>
-          <t>目前電腦設備故障，僅透過teams與IT人員報修聯絡。</t>
+      <c r="N69" s="60" t="inlineStr">
+        <is>
+          <t>電腦設備故障多透過 Teams 向資訊人員報修，未建置資訊服務需求單。</t>
         </is>
       </c>
       <c r="O69" s="3" t="inlineStr">
@@ -7267,9 +7276,9 @@
           <t>制度與程序</t>
         </is>
       </c>
-      <c r="E70" s="3" t="inlineStr">
-        <is>
-          <t>發生事故時因欠缺處理程序而耽誤或發生重工問題</t>
+      <c r="E70" s="61" t="inlineStr">
+        <is>
+          <t>發生事故時欠缺處理程序，致延誤或重工</t>
         </is>
       </c>
       <c r="F70" s="1" t="inlineStr">
@@ -7352,9 +7361,9 @@
           <t>系統復原</t>
         </is>
       </c>
-      <c r="E71" s="3" t="inlineStr">
-        <is>
-          <t>執行程式因異常中斷未能及時恢復，而使資料處理發生延遲、遺漏或不完整</t>
+      <c r="E71" s="61" t="inlineStr">
+        <is>
+          <t>執行程式異常中斷未能及時恢復，致資料處理延遲、遺漏或不完整</t>
         </is>
       </c>
       <c r="F71" s="1" t="inlineStr">
@@ -7397,9 +7406,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N71" s="52" t="inlineStr">
-        <is>
-          <t>未發生過，故未建置</t>
+      <c r="N71" s="60" t="inlineStr">
+        <is>
+          <t>實務上尚未發生，相關程序未建置</t>
         </is>
       </c>
       <c r="O71" s="3" t="inlineStr">
@@ -7437,9 +7446,9 @@
           <t>備份</t>
         </is>
       </c>
-      <c r="E72" s="3" t="inlineStr">
-        <is>
-          <t>公司發生災害因重要資料文件無備份而永遠遺失</t>
+      <c r="E72" s="61" t="inlineStr">
+        <is>
+          <t>災害發生時重要資料無備份而永久遺失</t>
         </is>
       </c>
       <c r="F72" s="1" t="inlineStr">
@@ -7517,14 +7526,14 @@
           <t>系統復原計畫制度及測試程序之控制作業</t>
         </is>
       </c>
-      <c r="D73" s="3" t="inlineStr">
-        <is>
-          <t>備份回復 / 制度與程序</t>
-        </is>
-      </c>
-      <c r="E73" s="3" t="inlineStr">
-        <is>
-          <t>備援資料檔（庫）因存放位置、版本或取用責任不明，而無法於系統復原或資料調復需求發生時及時取得</t>
+      <c r="D73" s="61" t="inlineStr">
+        <is>
+          <t>備份回復／制度與程序</t>
+        </is>
+      </c>
+      <c r="E73" s="61" t="inlineStr">
+        <is>
+          <t>備援資料存放位置、版本或取用責任不明，系統復原或調復時無法及時取得</t>
         </is>
       </c>
       <c r="F73" s="1" t="inlineStr">
@@ -7557,9 +7566,9 @@
           <t>人工</t>
         </is>
       </c>
-      <c r="L73" s="9" t="inlineStr">
-        <is>
-          <t>預防性制度</t>
+      <c r="L73" s="59" t="inlineStr">
+        <is>
+          <t>預防性控制</t>
         </is>
       </c>
       <c r="M73" s="30" t="inlineStr">
@@ -7607,9 +7616,9 @@
           <t>備份回復測試</t>
         </is>
       </c>
-      <c r="E74" s="3" t="inlineStr">
-        <is>
-          <t>系統復原因所需資源不完整或無法使用，而無法依預定方式及時完成</t>
+      <c r="E74" s="61" t="inlineStr">
+        <is>
+          <t>系統復原所需資源不完整或不可用，無法依預定方式及時完成復原</t>
         </is>
       </c>
       <c r="F74" s="1" t="inlineStr">
@@ -7692,9 +7701,9 @@
           <t>資訊設備保險</t>
         </is>
       </c>
-      <c r="E75" s="3" t="inlineStr">
-        <is>
-          <t>重要系統資源毀損致公司蒙受重大財務損失</t>
+      <c r="E75" s="61" t="inlineStr">
+        <is>
+          <t>重要系統資源毀損，致公司蒙受重大財務損失</t>
         </is>
       </c>
       <c r="F75" s="1" t="inlineStr">
@@ -7777,9 +7786,9 @@
           <t>資安政策</t>
         </is>
       </c>
-      <c r="E76" s="3" t="inlineStr">
-        <is>
-          <t>資訊安全作業因缺乏一致之規範及指引，而發生不符合公司安全要求之作業行為</t>
+      <c r="E76" s="61" t="inlineStr">
+        <is>
+          <t>資訊安全作業缺乏一致規範，發生不符公司安全要求之行為</t>
         </is>
       </c>
       <c r="F76" s="1" t="inlineStr">
@@ -7822,9 +7831,9 @@
           <t>持續</t>
         </is>
       </c>
-      <c r="N76" s="52" t="inlineStr">
-        <is>
-          <t>公司已向員工進行資安宣導配合 ISO 27001 的導入與輔導，已陸續增加宣導次數與內容以符合規範要求。</t>
+      <c r="N76" s="60" t="inlineStr">
+        <is>
+          <t>配合 ISO 27001 導入與輔導，已對員工進行資安宣導並增加宣導次數與內容。</t>
         </is>
       </c>
       <c r="O76" s="3" t="n"/>
@@ -7858,9 +7867,9 @@
           <t>資訊安全組織</t>
         </is>
       </c>
-      <c r="E77" s="3" t="inlineStr">
-        <is>
-          <t>資訊安全業務因權責歸屬不明或職能分散，而無法有效協調、執行及追蹤</t>
+      <c r="E77" s="61" t="inlineStr">
+        <is>
+          <t>資訊安全業務權責不明或職能分散，無法有效協調、執行及追蹤</t>
         </is>
       </c>
       <c r="F77" s="1" t="inlineStr">
@@ -7903,9 +7912,9 @@
           <t>持續</t>
         </is>
       </c>
-      <c r="N77" s="51" t="inlineStr">
-        <is>
-          <t>按公司政策"XXX"，公司之資訊部門""即為資安組織；資訊安全組織之最高負責人，由公司XXX兼任。</t>
+      <c r="N77" s="73" t="inlineStr">
+        <is>
+          <t>資訊單位兼任資安組織（政策名稱及最高負責人待確認）。</t>
         </is>
       </c>
       <c r="O77" s="3" t="n"/>
@@ -7939,9 +7948,9 @@
           <t>教育宣導與訓練</t>
         </is>
       </c>
-      <c r="E78" s="3" t="inlineStr">
-        <is>
-          <t>員工因資安意識及法規認知不足，而發生不符合公司資訊安全要求之行為</t>
+      <c r="E78" s="61" t="inlineStr">
+        <is>
+          <t>員工資安意識或法規認知不足，發生不符公司資訊安全要求之行為</t>
         </is>
       </c>
       <c r="F78" s="1" t="inlineStr">
@@ -7969,8 +7978,16 @@
           <t>公司應持續向全體員工宣導公司資安規定與相關法規。</t>
         </is>
       </c>
-      <c r="K78" s="9" t="n"/>
-      <c r="L78" s="9" t="n"/>
+      <c r="K78" s="59" t="inlineStr">
+        <is>
+          <t>人工</t>
+        </is>
+      </c>
+      <c r="L78" s="59" t="inlineStr">
+        <is>
+          <t>預防性控制</t>
+        </is>
+      </c>
       <c r="M78" s="30" t="inlineStr">
         <is>
           <t>TBC</t>
@@ -8016,9 +8033,9 @@
           <t>防毒掃描</t>
         </is>
       </c>
-      <c r="E79" s="3" t="inlineStr">
-        <is>
-          <t>公司伺服器及電腦因感染病毒或惡意程式，而發生系統異常、資料毀損或機密資料外洩</t>
+      <c r="E79" s="61" t="inlineStr">
+        <is>
+          <t>伺服器或電腦感染病毒或惡意程式，致系統異常、資料毀損或機密外洩</t>
         </is>
       </c>
       <c r="F79" s="1" t="inlineStr">
@@ -8061,9 +8078,9 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="N79" s="52" t="inlineStr">
-        <is>
-          <t>公司目前已使用防毒軟體，並由資訊人員定期手動更新。 &gt; TBC: 安裝在哪些設備上</t>
+      <c r="N79" s="60" t="inlineStr">
+        <is>
+          <t>已安裝防毒軟體，由資訊人員定期手動更新；涵蓋設備範圍待確認。</t>
         </is>
       </c>
       <c r="O79" s="3" t="n"/>
@@ -8092,14 +8109,14 @@
           <t>資通安全檢查之控制作業</t>
         </is>
       </c>
-      <c r="D80" s="3" t="inlineStr">
-        <is>
-          <t>防毒掃描 / 教育宣導與訓練</t>
-        </is>
-      </c>
-      <c r="E80" s="3" t="inlineStr">
-        <is>
-          <t>員工誤植惡意軟體程式引發公司重大資安事件</t>
+      <c r="D80" s="61" t="inlineStr">
+        <is>
+          <t>防毒掃描／教育宣導與訓練</t>
+        </is>
+      </c>
+      <c r="E80" s="61" t="inlineStr">
+        <is>
+          <t>員工誤用外來媒體植入惡意程式，引發重大資安事件</t>
         </is>
       </c>
       <c r="F80" s="1" t="inlineStr">
@@ -8177,14 +8194,14 @@
           <t>資通安全檢查之控制作業</t>
         </is>
       </c>
-      <c r="D81" s="3" t="inlineStr">
-        <is>
-          <t>制度與程序 / 資安事件處理</t>
-        </is>
-      </c>
-      <c r="E81" s="3" t="inlineStr">
-        <is>
-          <t>資安事件無法被即時排除與通報演變成公司重大資安事故</t>
+      <c r="D81" s="61" t="inlineStr">
+        <is>
+          <t>制度與程序／資安事件處理</t>
+        </is>
+      </c>
+      <c r="E81" s="61" t="inlineStr">
+        <is>
+          <t>資安事件未能即時排除與通報，演變成重大資安事故</t>
         </is>
       </c>
       <c r="F81" s="1" t="inlineStr">
@@ -8267,9 +8284,9 @@
           <t>防火牆管理</t>
         </is>
       </c>
-      <c r="E82" s="3" t="inlineStr">
-        <is>
-          <t>公司網路因保護措施不足而遭入侵滲透，造成機密與敏感資料洩漏</t>
+      <c r="E82" s="61" t="inlineStr">
+        <is>
+          <t>網路防護不足遭入侵滲透，造成機密與敏感資料洩漏</t>
         </is>
       </c>
       <c r="F82" s="1" t="inlineStr">
@@ -8292,9 +8309,9 @@
           <t>EC-110-07</t>
         </is>
       </c>
-      <c r="J82" s="3" t="inlineStr">
-        <is>
-          <t>公司應架設網路防護系統（包含防火牆及入侵偵測或保護系統）；任何設定或參數變更應取得資訓單位主管授權後，始得辦理。</t>
+      <c r="J82" s="61" t="inlineStr">
+        <is>
+          <t>公司應架設網路防護系統（含防火牆及入侵偵測或防護系統）；設定或參數變更應經資訊單位主管核准後辦理。</t>
         </is>
       </c>
       <c r="K82" s="9" t="inlineStr">
@@ -8352,9 +8369,9 @@
           <t>遠端存取控制</t>
         </is>
       </c>
-      <c r="E83" s="3" t="inlineStr">
-        <is>
-          <t>公司內部網路遭未經授權之遠端連線存取，而發生系統入侵或機密資料外洩</t>
+      <c r="E83" s="61" t="inlineStr">
+        <is>
+          <t>未經授權之遠端連線存取內部網路，致系統入侵或機密外洩</t>
         </is>
       </c>
       <c r="F83" s="1" t="inlineStr">
@@ -8437,9 +8454,9 @@
           <t>防火牆管理</t>
         </is>
       </c>
-      <c r="E84" s="3" t="inlineStr">
-        <is>
-          <t>未辨識或排除網路異常連線致網路防火牆被攻破失效</t>
+      <c r="E84" s="61" t="inlineStr">
+        <is>
+          <t>網路異常連線未辨識或排除，致防火牆防護失效</t>
         </is>
       </c>
       <c r="F84" s="1" t="inlineStr">
@@ -8517,14 +8534,14 @@
           <t>委外服務之控制作業</t>
         </is>
       </c>
-      <c r="D85" s="3" t="inlineStr">
-        <is>
-          <t>資訊委外服務 / 供應商管理</t>
-        </is>
-      </c>
-      <c r="E85" s="3" t="inlineStr">
-        <is>
-          <t>委外服務機構因資格或服務能力不符公司需求，而影響委外服務品質及資訊資產安全</t>
+      <c r="D85" s="61" t="inlineStr">
+        <is>
+          <t>資訊委外服務／供應商管理</t>
+        </is>
+      </c>
+      <c r="E85" s="61" t="inlineStr">
+        <is>
+          <t>委外機構資格或能力不符需求，影響服務品質及資訊資產安全</t>
         </is>
       </c>
       <c r="F85" s="1" t="inlineStr">
@@ -8567,9 +8584,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N85" s="52" t="inlineStr">
-        <is>
-          <t>專業性機器設備、軟體、IP等之採購，請購單位填寫EasyFlow「請購單」後，依核決權限經核准後，由請購單位依其專業知識尋找供應商，並提供相關資料予採購單位進行詢價、比價、議價。</t>
+      <c r="N85" s="60" t="inlineStr">
+        <is>
+          <t>專業設備、軟體、IP 等請購，由請購單位填寫 EasyFlow「請購單」經核決後，由請購單位尋找供應商，再交採購單位詢比議價。</t>
         </is>
       </c>
       <c r="O85" s="3" t="n"/>
@@ -8598,14 +8615,14 @@
           <t>委外服務之控制作業</t>
         </is>
       </c>
-      <c r="D86" s="3" t="inlineStr">
-        <is>
-          <t>資訊委外服務 / 合約與外包</t>
-        </is>
-      </c>
-      <c r="E86" s="3" t="inlineStr">
-        <is>
-          <t>委外廠商因服務權責及存取範圍不明，而逾越授權範圍存取公司資訊設備或洩漏機密資料</t>
+      <c r="D86" s="61" t="inlineStr">
+        <is>
+          <t>資訊委外服務／合約與外包</t>
+        </is>
+      </c>
+      <c r="E86" s="61" t="inlineStr">
+        <is>
+          <t>委外廠商服務權責或存取範圍不明，逾權存取設備或洩漏機密</t>
         </is>
       </c>
       <c r="F86" s="1" t="inlineStr">
@@ -8648,9 +8665,9 @@
           <t>不定期</t>
         </is>
       </c>
-      <c r="N86" s="52" t="inlineStr">
-        <is>
-          <t>以於委外廠商簽訂合約時包含資訊安全政策規範之內容。</t>
+      <c r="N86" s="60" t="inlineStr">
+        <is>
+          <t>與委外廠商簽訂合約時，納入資訊安全相關規範。</t>
         </is>
       </c>
       <c r="O86" s="3" t="n"/>
@@ -8679,9 +8696,9 @@
           <t>委外服務之控制作業</t>
         </is>
       </c>
-      <c r="D87" s="21" t="inlineStr">
-        <is>
-          <t>資訊委外服務 / 合約與外包</t>
+      <c r="D87" s="77" t="inlineStr">
+        <is>
+          <t>資訊委外服務／合約與外包</t>
         </is>
       </c>
       <c r="E87" s="37" t="inlineStr">
@@ -8729,9 +8746,9 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="N87" s="69" t="inlineStr">
-        <is>
-          <t>未實施 &gt; 實務上不常發生 要硬加嗎 TBD: 實務上如何執行</t>
+      <c r="N87" s="78" t="inlineStr">
+        <is>
+          <t>未實施對委外廠商之安全及隱私控制查核（實務執行方式待確認）。</t>
         </is>
       </c>
       <c r="O87" s="21" t="inlineStr">
@@ -8854,9 +8871,9 @@
           <t>公開資訊申報</t>
         </is>
       </c>
-      <c r="E89" s="22" t="inlineStr">
-        <is>
-          <t>上傳錯誤或漏失申報資訊，導致公司蒙受主管機關裁罰</t>
+      <c r="E89" s="77" t="inlineStr">
+        <is>
+          <t>上傳錯誤或漏報公開資訊，致主管機關裁罰</t>
         </is>
       </c>
       <c r="F89" s="19" t="inlineStr">

</xml_diff>